<commit_message>
node version is fix for node 18.20
</commit_message>
<xml_diff>
--- a/Backend/reports/Daily_Disbursement_Case_Count_2026-10-09.xlsx
+++ b/Backend/reports/Daily_Disbursement_Case_Count_2026-10-09.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1486" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1606" uniqueCount="811">
   <si>
     <t>Daily Partner-wise Disbursement Case Count Report</t>
   </si>
@@ -50,7 +50,7 @@
     <t>Total Disbursed Cases</t>
   </si>
   <si>
-    <t>Disbursed Case Details (09-10-2026) - Total: 367 Cases</t>
+    <t>Disbursed Case Details (09-10-2026) - Total: 397 Cases</t>
   </si>
   <si>
     <t>LAN</t>
@@ -341,6 +341,12 @@
     <t>628216295889</t>
   </si>
   <si>
+    <t>FINEW126666</t>
+  </si>
+  <si>
+    <t>628217369877</t>
+  </si>
+  <si>
     <t>LDF1011969</t>
   </si>
   <si>
@@ -365,6 +371,12 @@
     <t>628212785910</t>
   </si>
   <si>
+    <t>QML1017511</t>
+  </si>
+  <si>
+    <t>628217359896</t>
+  </si>
+  <si>
     <t>QML1020441</t>
   </si>
   <si>
@@ -377,6 +389,12 @@
     <t>628211608019</t>
   </si>
   <si>
+    <t>QML1023567</t>
+  </si>
+  <si>
+    <t>628217460678</t>
+  </si>
+  <si>
     <t>QML1027147</t>
   </si>
   <si>
@@ -401,6 +419,12 @@
     <t>628208330407</t>
   </si>
   <si>
+    <t>QML1033871</t>
+  </si>
+  <si>
+    <t>628218465876</t>
+  </si>
+  <si>
     <t>QML1034324</t>
   </si>
   <si>
@@ -479,6 +503,12 @@
     <t>628214967058</t>
   </si>
   <si>
+    <t>QML1037196</t>
+  </si>
+  <si>
+    <t>628217426440</t>
+  </si>
+  <si>
     <t>QML1038187</t>
   </si>
   <si>
@@ -527,6 +557,12 @@
     <t>628212787383</t>
   </si>
   <si>
+    <t>QML1038399</t>
+  </si>
+  <si>
+    <t>628217444012</t>
+  </si>
+  <si>
     <t>QML1038453</t>
   </si>
   <si>
@@ -719,6 +755,12 @@
     <t>628215171726</t>
   </si>
   <si>
+    <t>QML1039094</t>
+  </si>
+  <si>
+    <t>628217406308</t>
+  </si>
+  <si>
     <t>QML1039107</t>
   </si>
   <si>
@@ -767,6 +809,12 @@
     <t>628210494575</t>
   </si>
   <si>
+    <t>RML10103663</t>
+  </si>
+  <si>
+    <t>628218466065</t>
+  </si>
+  <si>
     <t>RML10104452</t>
   </si>
   <si>
@@ -851,6 +899,12 @@
     <t>628212789349</t>
   </si>
   <si>
+    <t>RML10115474</t>
+  </si>
+  <si>
+    <t>628217438519</t>
+  </si>
+  <si>
     <t>RML10115551</t>
   </si>
   <si>
@@ -1127,6 +1181,12 @@
     <t>628208312140</t>
   </si>
   <si>
+    <t>RML10119876</t>
+  </si>
+  <si>
+    <t>628217395658</t>
+  </si>
+  <si>
     <t>RML10119886</t>
   </si>
   <si>
@@ -1157,6 +1217,12 @@
     <t>628208325717</t>
   </si>
   <si>
+    <t>RML10119995</t>
+  </si>
+  <si>
+    <t>628217408360</t>
+  </si>
+  <si>
     <t>RML10120006</t>
   </si>
   <si>
@@ -1649,6 +1715,12 @@
     <t>628212780585</t>
   </si>
   <si>
+    <t>RML10120886</t>
+  </si>
+  <si>
+    <t>628217400276</t>
+  </si>
+  <si>
     <t>RML10120891</t>
   </si>
   <si>
@@ -2135,12 +2207,24 @@
     <t>628217329067</t>
   </si>
   <si>
+    <t>RML10121310</t>
+  </si>
+  <si>
+    <t>628217362772</t>
+  </si>
+  <si>
     <t>RML10121313</t>
   </si>
   <si>
     <t>628216310877</t>
   </si>
   <si>
+    <t>RML10121314</t>
+  </si>
+  <si>
+    <t>628217398353</t>
+  </si>
+  <si>
     <t>RML10121323</t>
   </si>
   <si>
@@ -2177,6 +2261,12 @@
     <t>628216313244</t>
   </si>
   <si>
+    <t>RML10121343</t>
+  </si>
+  <si>
+    <t>628217442896</t>
+  </si>
+  <si>
     <t>RML10121345</t>
   </si>
   <si>
@@ -2207,6 +2297,84 @@
     <t>628217344820</t>
   </si>
   <si>
+    <t>RML10121376</t>
+  </si>
+  <si>
+    <t>628217351484</t>
+  </si>
+  <si>
+    <t>RML10121391</t>
+  </si>
+  <si>
+    <t>628217358619</t>
+  </si>
+  <si>
+    <t>RML10121393</t>
+  </si>
+  <si>
+    <t>628217361963</t>
+  </si>
+  <si>
+    <t>RML10121396</t>
+  </si>
+  <si>
+    <t>628217358839</t>
+  </si>
+  <si>
+    <t>RML10121397</t>
+  </si>
+  <si>
+    <t>628217358781</t>
+  </si>
+  <si>
+    <t>RML10121408</t>
+  </si>
+  <si>
+    <t>628217399298</t>
+  </si>
+  <si>
+    <t>RML10121414</t>
+  </si>
+  <si>
+    <t>628217395829</t>
+  </si>
+  <si>
+    <t>RML10121435</t>
+  </si>
+  <si>
+    <t>628217453267</t>
+  </si>
+  <si>
+    <t>RML10121440</t>
+  </si>
+  <si>
+    <t>628217425118</t>
+  </si>
+  <si>
+    <t>RML10121441</t>
+  </si>
+  <si>
+    <t>628217431185</t>
+  </si>
+  <si>
+    <t>RML10121457</t>
+  </si>
+  <si>
+    <t>628217448210</t>
+  </si>
+  <si>
+    <t>RML10121465</t>
+  </si>
+  <si>
+    <t>628217448402</t>
+  </si>
+  <si>
+    <t>RML10121477</t>
+  </si>
+  <si>
+    <t>628217464086</t>
+  </si>
+  <si>
     <t>RML1051359</t>
   </si>
   <si>
@@ -2243,6 +2411,12 @@
     <t>628213877775</t>
   </si>
   <si>
+    <t>RML1089340</t>
+  </si>
+  <si>
+    <t>628217398187</t>
+  </si>
+  <si>
     <t>RML1090805</t>
   </si>
   <si>
@@ -2253,6 +2427,12 @@
   </si>
   <si>
     <t>628210499957</t>
+  </si>
+  <si>
+    <t>RML1095501</t>
+  </si>
+  <si>
+    <t>628217400362</t>
   </si>
   <si>
     <t>RML1096608</t>
@@ -2869,7 +3049,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="7">
-        <v>254</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2880,7 +3060,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="10">
-        <v>62</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2891,7 +3071,7 @@
         <v>7</v>
       </c>
       <c r="C7" s="7">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2924,7 +3104,7 @@
         <v>11</v>
       </c>
       <c r="C10" s="13">
-        <v>367</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>
@@ -2939,7 +3119,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E369"/>
+  <dimension ref="A1:E399"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -3765,7 +3945,7 @@
         <v>109</v>
       </c>
       <c r="C49" s="18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D49" s="17" t="s">
         <v>17</v>
@@ -3833,7 +4013,7 @@
         <v>117</v>
       </c>
       <c r="C53" s="18" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D53" s="17" t="s">
         <v>17</v>
@@ -4887,7 +5067,7 @@
         <v>241</v>
       </c>
       <c r="C115" s="18" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D115" s="17" t="s">
         <v>17</v>
@@ -4904,7 +5084,7 @@
         <v>243</v>
       </c>
       <c r="C116" s="20" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D116" s="19" t="s">
         <v>17</v>
@@ -4921,7 +5101,7 @@
         <v>245</v>
       </c>
       <c r="C117" s="18" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D117" s="17" t="s">
         <v>17</v>
@@ -4938,7 +5118,7 @@
         <v>247</v>
       </c>
       <c r="C118" s="20" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D118" s="19" t="s">
         <v>17</v>
@@ -4955,7 +5135,7 @@
         <v>249</v>
       </c>
       <c r="C119" s="18" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D119" s="17" t="s">
         <v>17</v>
@@ -4972,7 +5152,7 @@
         <v>251</v>
       </c>
       <c r="C120" s="20" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D120" s="19" t="s">
         <v>17</v>
@@ -4989,7 +5169,7 @@
         <v>253</v>
       </c>
       <c r="C121" s="18" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D121" s="17" t="s">
         <v>17</v>
@@ -9205,13 +9385,523 @@
         <v>749</v>
       </c>
       <c r="C369" s="18" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D369" s="17" t="s">
         <v>17</v>
       </c>
       <c r="E369" s="18" t="s">
         <v>750</v>
+      </c>
+    </row>
+    <row r="370" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A370" s="19">
+        <v>368</v>
+      </c>
+      <c r="B370" s="20" t="s">
+        <v>751</v>
+      </c>
+      <c r="C370" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D370" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E370" s="20" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="371" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A371" s="17">
+        <v>369</v>
+      </c>
+      <c r="B371" s="18" t="s">
+        <v>753</v>
+      </c>
+      <c r="C371" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D371" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E371" s="18" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="372" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A372" s="19">
+        <v>370</v>
+      </c>
+      <c r="B372" s="20" t="s">
+        <v>755</v>
+      </c>
+      <c r="C372" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D372" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E372" s="20" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="373" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A373" s="17">
+        <v>371</v>
+      </c>
+      <c r="B373" s="18" t="s">
+        <v>757</v>
+      </c>
+      <c r="C373" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D373" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E373" s="18" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="374" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A374" s="19">
+        <v>372</v>
+      </c>
+      <c r="B374" s="20" t="s">
+        <v>759</v>
+      </c>
+      <c r="C374" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D374" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E374" s="20" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="375" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A375" s="17">
+        <v>373</v>
+      </c>
+      <c r="B375" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="C375" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D375" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E375" s="18" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="376" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A376" s="19">
+        <v>374</v>
+      </c>
+      <c r="B376" s="20" t="s">
+        <v>763</v>
+      </c>
+      <c r="C376" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D376" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E376" s="20" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="377" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A377" s="17">
+        <v>375</v>
+      </c>
+      <c r="B377" s="18" t="s">
+        <v>765</v>
+      </c>
+      <c r="C377" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D377" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E377" s="18" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="378" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A378" s="19">
+        <v>376</v>
+      </c>
+      <c r="B378" s="20" t="s">
+        <v>767</v>
+      </c>
+      <c r="C378" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D378" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E378" s="20" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="379" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A379" s="17">
+        <v>377</v>
+      </c>
+      <c r="B379" s="18" t="s">
+        <v>769</v>
+      </c>
+      <c r="C379" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D379" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E379" s="18" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="380" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A380" s="19">
+        <v>378</v>
+      </c>
+      <c r="B380" s="20" t="s">
+        <v>771</v>
+      </c>
+      <c r="C380" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D380" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E380" s="20" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="381" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A381" s="17">
+        <v>379</v>
+      </c>
+      <c r="B381" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="C381" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D381" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E381" s="18" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="382" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A382" s="19">
+        <v>380</v>
+      </c>
+      <c r="B382" s="20" t="s">
+        <v>775</v>
+      </c>
+      <c r="C382" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D382" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E382" s="20" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="383" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A383" s="17">
+        <v>381</v>
+      </c>
+      <c r="B383" s="18" t="s">
+        <v>777</v>
+      </c>
+      <c r="C383" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D383" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E383" s="18" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="384" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A384" s="19">
+        <v>382</v>
+      </c>
+      <c r="B384" s="20" t="s">
+        <v>779</v>
+      </c>
+      <c r="C384" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D384" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E384" s="20" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="385" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A385" s="17">
+        <v>383</v>
+      </c>
+      <c r="B385" s="18" t="s">
+        <v>781</v>
+      </c>
+      <c r="C385" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D385" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E385" s="18" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="386" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A386" s="19">
+        <v>384</v>
+      </c>
+      <c r="B386" s="20" t="s">
+        <v>783</v>
+      </c>
+      <c r="C386" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D386" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E386" s="20" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="387" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A387" s="17">
+        <v>385</v>
+      </c>
+      <c r="B387" s="18" t="s">
+        <v>785</v>
+      </c>
+      <c r="C387" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D387" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E387" s="18" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="388" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A388" s="19">
+        <v>386</v>
+      </c>
+      <c r="B388" s="20" t="s">
+        <v>787</v>
+      </c>
+      <c r="C388" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D388" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E388" s="20" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="389" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A389" s="17">
+        <v>387</v>
+      </c>
+      <c r="B389" s="18" t="s">
+        <v>789</v>
+      </c>
+      <c r="C389" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D389" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E389" s="18" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="390" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A390" s="19">
+        <v>388</v>
+      </c>
+      <c r="B390" s="20" t="s">
+        <v>791</v>
+      </c>
+      <c r="C390" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D390" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E390" s="20" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="391" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A391" s="17">
+        <v>389</v>
+      </c>
+      <c r="B391" s="18" t="s">
+        <v>793</v>
+      </c>
+      <c r="C391" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D391" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E391" s="18" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="392" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A392" s="19">
+        <v>390</v>
+      </c>
+      <c r="B392" s="20" t="s">
+        <v>795</v>
+      </c>
+      <c r="C392" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D392" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E392" s="20" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="393" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A393" s="17">
+        <v>391</v>
+      </c>
+      <c r="B393" s="18" t="s">
+        <v>797</v>
+      </c>
+      <c r="C393" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D393" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E393" s="18" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="394" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A394" s="19">
+        <v>392</v>
+      </c>
+      <c r="B394" s="20" t="s">
+        <v>799</v>
+      </c>
+      <c r="C394" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D394" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E394" s="20" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="395" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A395" s="17">
+        <v>393</v>
+      </c>
+      <c r="B395" s="18" t="s">
+        <v>801</v>
+      </c>
+      <c r="C395" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D395" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E395" s="18" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="396" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A396" s="19">
+        <v>394</v>
+      </c>
+      <c r="B396" s="20" t="s">
+        <v>803</v>
+      </c>
+      <c r="C396" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D396" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E396" s="20" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="397" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A397" s="17">
+        <v>395</v>
+      </c>
+      <c r="B397" s="18" t="s">
+        <v>805</v>
+      </c>
+      <c r="C397" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D397" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E397" s="18" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="398" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A398" s="19">
+        <v>396</v>
+      </c>
+      <c r="B398" s="20" t="s">
+        <v>807</v>
+      </c>
+      <c r="C398" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D398" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E398" s="20" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="399" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A399" s="17">
+        <v>397</v>
+      </c>
+      <c r="B399" s="18" t="s">
+        <v>809</v>
+      </c>
+      <c r="C399" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D399" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E399" s="18" t="s">
+        <v>810</v>
       </c>
     </row>
   </sheetData>

</xml_diff>